<commit_message>
Refactor to standalone offline Excel extraction tool and anonymize project names
</commit_message>
<xml_diff>
--- a/telecom_extracted_requirements.xlsx
+++ b/telecom_extracted_requirements.xlsx
@@ -480,7 +480,8 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Clause or Drawing No.</t>
+          <t>Clause or
+Drawing No.</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -547,12 +548,12 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea.pdf</t>
+          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>F. TERMINAL POINTS / Table.1 / Location: Simhadri / S.No.11</t>
+          <t>F. TERMINAL POINTS / Table.1 / Location: Site Alpha / S.No.11</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
@@ -579,12 +580,12 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea.pdf</t>
+          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>F. TERMINAL POINTS / Location: Pudimadaka / S.No.7</t>
+          <t>F. TERMINAL POINTS / Location: Site Beta / S.No.7</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
@@ -611,7 +612,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea.pdf</t>
+          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -643,7 +644,7 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea.pdf</t>
+          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -675,7 +676,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea.pdf</t>
+          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -707,7 +708,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea.pdf</t>
+          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -739,7 +740,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea.pdf</t>
+          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -771,7 +772,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea.pdf</t>
+          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
@@ -796,14 +797,14 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Dual redundant 10kVA UPS system with Ni-Cd battery bank providing 3 hours backup for DCS/PLC and instrumentation loads at Simhadri CO2 Capture Block.</t>
+          <t>Dual redundant 10kVA UPS system with Ni-Cd battery bank providing 3 hours backup for DCS/PLC and instrumentation loads at Site Alpha CO2 Capture Block.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea.pdf</t>
+          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -823,19 +824,19 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>The bidder shall provide remote monitoring (read-only data flow) for the CO2 capture plant (located at Simhadri) at Pudimadaka. The Pudimadaka standalone monitoring system shall be non-control, with no interface to plant control systems, and will follow cybersecurity-driven network isolation with secure, standardized communication (e.g., OPC) to ensure reliable data monitoring. The system shall include historian with a minimum storage capacity of two months.</t>
+          <t>The bidder shall provide remote monitoring (read-only data flow) for the CO2 capture plant (located at Site Alpha) at Site Beta. The Site Beta standalone monitoring system shall be non-control, with no interface to plant control systems, and will follow cybersecurity-driven network isolation with secure, standardized communication (e.g., OPC) to ensure reliable data monitoring. The system shall include historian with a minimum storage capacity of two months.</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Establish a read-only remote monitoring interface from Simhadri to Pudimadaka using OPC communication, including cybersecurity network isolation and a historian with minimum 2 months storage.</t>
+          <t>Establish a read-only remote monitoring interface from Site Alpha to Site Beta using OPC communication, including cybersecurity network isolation and a historian with minimum 2 months storage.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea.pdf</t>
+          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
@@ -867,7 +868,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea.pdf</t>
+          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -899,7 +900,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea.pdf</t>
+          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
@@ -931,7 +932,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea.pdf</t>
+          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -963,7 +964,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea.pdf</t>
+          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
@@ -995,7 +996,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea.pdf</t>
+          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -1027,7 +1028,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea.pdf</t>
+          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
@@ -1059,7 +1060,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea.pdf</t>
+          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -1091,7 +1092,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea.pdf</t>
+          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
@@ -1123,7 +1124,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea.pdf</t>
+          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -1155,7 +1156,7 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea.pdf</t>
+          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
@@ -1187,7 +1188,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea.pdf</t>
+          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -1219,7 +1220,7 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea.pdf</t>
+          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
@@ -1251,7 +1252,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea.pdf</t>
+          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -1283,7 +1284,7 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea.pdf</t>
+          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
@@ -1315,7 +1316,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea.pdf</t>
+          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -1347,7 +1348,7 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea.pdf</t>
+          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
@@ -1379,7 +1380,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea.pdf</t>
+          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -1411,7 +1412,7 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea.pdf</t>
+          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
@@ -1443,7 +1444,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea.pdf</t>
+          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
@@ -1453,7 +1454,7 @@
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>42-43</t>
+          <t>42</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
@@ -1475,7 +1476,7 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea.pdf</t>
+          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
@@ -1507,7 +1508,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea.pdf</t>
+          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -1539,7 +1540,7 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea.pdf</t>
+          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
@@ -1571,7 +1572,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea.pdf</t>
+          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
@@ -1581,7 +1582,7 @@
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>43-44</t>
+          <t>43</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
@@ -1603,7 +1604,7 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea.pdf</t>
+          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
@@ -1635,7 +1636,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea.pdf</t>
+          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
@@ -1667,7 +1668,7 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea.pdf</t>
+          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
@@ -1699,7 +1700,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea.pdf</t>
+          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
@@ -1731,7 +1732,7 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea.pdf</t>
+          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
@@ -1746,24 +1747,24 @@
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>Control Room Civil Design - Simhadri</t>
+          <t>Control Room Civil Design - Site Alpha</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>Electrical cum Control Room for Carbon capture plant at Simadhari: A RCC / pre-engineered structural steel Building (25m X 12m) tentative shall be provided. The building shall be covered from all sides. The Electrical Room shall accommodate, LT PMCC Panels, Dry Type Transformer (if applicable), VFD Transformers (if applicable), 220V DCFB, LDB, WDB. and UPS, UPS DCDB, UPS battery and operator cabin etc. as per functional requirement. However, final size of Switchgear room, Control room, individual room, partition, doors, windows, rolling shutter etc shall be finalized at the stage of detail engineering with the approval of NTPC. Control room, meeting room, office space with toilet, pantry, staircase etc., shall be provided with sufficient lighting, ceiling / wall mounted fans, office furniture (tables, chairs etc of reputed make) etc. Individual control room, meeting room, office space shall be able to house 5-8 people for regular operational requirement. Control Room shall be Air conditioned. The control shall accommodate all the equipment as mentioned in Electrical and C&amp;I chapter. The firefighting system shall be provided as per norms.</t>
+          <t>Electrical cum Control Room for Carbon capture plant at Site Alpha: A RCC / pre-engineered structural steel Building (25m X 12m) tentative shall be provided. The building shall be covered from all sides. The Electrical Room shall accommodate, LT PMCC Panels, Dry Type Transformer (if applicable), VFD Transformers (if applicable), 220V DCFB, LDB, WDB. and UPS, UPS DCDB, UPS battery and operator cabin etc. as per functional requirement. However, final size of Switchgear room, Control room, individual room, partition, doors, windows, rolling shutter etc shall be finalized at the stage of detail engineering with the approval of Client. Control room, meeting room, office space with toilet, pantry, staircase etc., shall be provided with sufficient lighting, ceiling / wall mounted fans, office furniture (tables, chairs etc of reputed make) etc. Individual control room, meeting room, office space shall be able to house 5-8 people for regular operational requirement. Control Room shall be Air conditioned. The control shall accommodate all the equipment as mentioned in Electrical and C&amp;I chapter. The firefighting system shall be provided as per norms.</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>Tentative 25x12m air-conditioned building at Simhadri to house C&amp;I and electrical systems, including UPS systems, batteries, and the operator cabin.</t>
+          <t>Tentative 25x12m air-conditioned building at Site Alpha to house C&amp;I and electrical systems, including UPS systems, batteries, and the operator cabin.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea.pdf</t>
+          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
@@ -1778,17 +1779,17 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>Control Room Civil Design - Pudimadaka</t>
+          <t>Control Room Civil Design - Site Beta</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>Electrical cum Control Room for Urea Plant at Pudimadka shall be as mentioned in technical Specification (Part-B). Bidder shall be free to locate civil structures including control room in a manner to avoid blast proof constructions. However, compliance of OISD and other relevant statutory and mandatory requirements shall be ensured.</t>
+          <t>Electrical cum Control Room for Urea Plant at Site Beta shall be as mentioned in technical Specification (Part-B). Bidder shall be free to locate civil structures including control room in a manner to avoid blast proof constructions. Client...</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>Pudimadaka Control Room civil design specification, with layout flexibility to avoid blast-proof construction while maintaining OISD compliance.</t>
+          <t>Site Beta Control Room civil design specification, with layout flexibility to avoid blast-proof construction while maintaining OISD compliance.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix openpyxl NameError and status polling race condition in web UI
</commit_message>
<xml_diff>
--- a/telecom_extracted_requirements.xlsx
+++ b/telecom_extracted_requirements.xlsx
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F42"/>
+  <dimension ref="A1:F29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -516,1280 +516,864 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Part_B3_Technical_Specification_CO2_Urea_1001_2000</t>
+          <t>Part_B1_Technical_Specification_CO2_Urea_1_500</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>B773-000-16-50-DS-0024, PLANT COMMUNICATION SYSTEM DATA SHEET</t>
+          <t>B773-000-83-41-LE-T-9902</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>108</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>PLANT COMMUNICATION SYSTEM DATA SHEE</t>
+          <t>OT Cybersecurity &amp; Network</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>C. Power Supply Type: UPS</t>
+          <t>| 2 een Click on the Document Title to go to that section of the document Table of Contents Document Number Document Title Number AnnexureA-B773- A SCOPE OF WORK AND SUPPLY (ANNEX-A-Static Equipment) 412 000-80-42-SOW- 9902 Annexure-C B773- |A SCOPE OF WORK/SUPPLY ANNEXURE-C: ROTATING 425 000-80-42-SOW- EQUIPMENT 9902 B773-000-80-42- eo | Scope of Works-Package Equipment SOW-9902 B773-00-000-19-41- eo | CONSTRUCTION SUPERVISION AND MANAGEMENT BY EPC 0002 CONTRACTOR B773-000-16-51-SP- B | Job Specifications (Instrumentation) 9902 B773-000-16-50-SP- JOB SPECIFICATION (ELECTRICAL) 9900 REV A B773-000-16-50-SP- B JOB SPECIFICATIONS 9902 B773-000-16-50-SP- JOB SPECIFICATION 8502 B773-000-16-50-SP- JOB SPECIFICATIONS 8501 B773-000-80-44-SP- A408 SPECIFICATION FOR ELECTRIC BOILER 3001 REV- 0 B773-000-16-51-SP- Job Specification for OT Cybersecurity Instrumentation 0001 Anexxure-A-B773- JOB SPECIFICATIONS (Annexure-A-Static Equipment) 000-80-42-SP-9902 Annexure-C B773- A 08 SPECIFICATION ANNEXURE-C: ROTATING EQUIPMENT 000-80-42-SP-9902 B773-000-80-42-SP- eo | Job Specification-Package Equipment 9902 B773-000-81-45-DS- DATA SHEET (HR) 4824 B773-000-81-45-DS- DATA SHEET (HB) 4825 B773-000-81-45-DS- DATA SHEET (LV) 4826 B773-000-81-45-DS- DATA SHEET (1000 GPM WFM) 4827 B773-000-81-45-DS- DATA SHEET (2000 GPM WFM) | 986 4828 B773-000-81-45-DS- DATA SHEET (HVLRM) 4829 B773-000-81-45-DS- DATA SHEET (MVS) 4000 4830 B773-000-81-45-DS- DATA SHEET (HVS) 1001 4831 B773-000-81-45-DS- DATA SHEET (DV) 1002 4832 B773-000-81-45-DS- DATA SHEET (RO) 1003 4833 B773-000-16-50-DS- DATA SHEET 1004 0001 B773-000-16-50-DS- DATA SHEET 1007 0002 B773-000-16-50-DS- DATA SHEET 1008 0003 Paae 3 of 7525 : B773-000-83-41-LE-T-9902 :Rev.B</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Backup Time Requirement for Telecom Power Supply, To be confirmed.</t>
+          <t>Verbatim specification requirement extracted dynamically.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea</t>
+          <t>Part_B1_Technical_Specification_CO2_Urea_1_500</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>F. TERMINAL POINTS / Table.1 / Location: Site Alpha / S.No.11</t>
+          <t>B773-000-83-41-LE-T-9902</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>6</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Security/CISF Control Room distance</t>
+          <t>Telecom Specifications</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Distance of CO2 Capture Plant from nearby Security/CISF Control Room '≥3000 meter</t>
+          <t>ere se Click on the Document Title to go to that section of the document Table of Contents Document Number Document Title Number Annexure-I-VL-9902- |A Storage Tank Contractor List 1626 Storage Tank Contractor List B773-000-16-50-VL- A VENDOR LIST 1628 9902 B773-000-16-43-VL- A VENDOR LIST (PIPING) FOR 150 TPD GREEN UREA 1715 9902 COMPLEX B773-000-80-42-VL- eo | Sub Vendor List-Package Equipment 1855 9902 Instrumentation B |Vendor List Instrumentation for B773 1858 Vendor List. B773-000-16-50- SINGLE LINE DIAGRAM 2012 0001 B773-000-81-45-0- OVERALL PLOT PLAN 2013 0001 B773-000-0341- R&amp;D INPUT 2014 SOW-9902 B773-6-44-0005-A1_|A _ [ANNEXURE-| TO PMS (GENERAL NOTES 2031 B773-6-44-0005-A2_ |A __— [ANNEXURE-I| TO PMS (EXTRACTS 2044 B773-6-44-0005 PIPING MATERIAL SPECIFICATIONS 2062 B773-6-44-0006-A1_|A ___— [ANNEXURE-I TO VMS (GENERAL NOTES 2274 B773-6-44-0006-A2_|A __—_—[ANNEXURE-II TO VMS (EXTRACTS 2280 B773-6-44-0006 [A _—_| VALVE MATERIAL SPECIFICATIONS 2300 B773-000-81-47- eo | GEOTECHNICAL DATA FOR 150TPD GREEN UREA PROJECT 2618 GTD-9902 B773-000-81-46-SP- B MISCELLANEOUS 2631 9902 Annexure-A B773- Standard Specification List (Annex-A-Static Equipment) 2646 000-80-42-LSP-9902 Annexure-A B773- SPARE LIST (ANNEX-A- Static Equipment) 2650 000-80-42-SL-9902 Annexure-A-B773- Standard Drawing List (Annex-A-Static Equipment) 2654 000-80-42-LL-9902 INSPECTION AND INSPECTION AND TEST PLAN (PIPING) FOR 150 TPD GREEN 2658 TEST PLAN UREA COMPLEX PIPING STANDARD PIPING STANDARD SPECIFICATIONS FOR 150 TPD GREEN 2743 SPECIFICATIONS UREA COMPLEX STANDARDS(PIPIN PIPING STANDARDS FOR 150 TPD GREEN UREA COMPLEX 3293 G Annexure-3 A Instrumentation MTO Blank Format 3344 _ Instrumentation MTO Blank Format Annexure-4_ Blank |A Blank Instrument datasheets format 3348 Instrument datasheets format B773-000-16-51-IOF-B IO Summary Blank Format 3416 7309 B773-000-16-51- B List of Engineering / Installation Standards (Instrumentation) 3419 MD01_9902 B773-000-16-51-SP- B Inspection and Test Plant List (Instrumentation) 3491 1001 9902 B773-000-16-51-SP- B Standard Specifications List (Instrumentation) 3686 1002 9902 B773-000-16-51-SP- B | List of Drawings (Instrumentation) 4363 1003 9902 Paae 6 of 7525 : B773-000-83-41-LE-T-9902 :Rev.B</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Physical security interface distance. Requirement column is verbatim table text only.</t>
+          <t>Verbatim specification requirement extracted dynamically.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea</t>
+          <t>Part_B1_Technical_Specification_CO2_Urea_1_500</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>F. TERMINAL POINTS / Location: Site Beta / S.No.7</t>
+          <t>B773-000-79-41-ODB-1001, Preparation of specification for LEL, gas like hydrogen and ammonia detectors and providing the same at suitable locations. - Finalizing vendor data /detailed engineering dependent fire case loads and finalizing corresponding relief valve inlet and outlet line sizes.</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>Page 69</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Security/CISF Control Room distance</t>
+          <t>CCTV Surveillance System</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Distance of Urea Plant B/L from nearby Security/CISF Control Room. '1000 meter</t>
+          <t>6. Surveillance camera for monitoring process plant asset, critical stacks, flare &amp; Security to be provided.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Physical security interface distance. Requirement column is verbatim table text only.</t>
+          <t>Verbatim specification requirement extracted dynamically.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea</t>
+          <t>Part_B1_Technical_Specification_CO2_Urea_1_500</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>A. Technical Specification – Mechanical / 2.g / NB-3</t>
+          <t>B773-79-41-PCS-01, Preparation of specification for LEL, gas like hydrogen and ammonia detectors and providing the same at suitable locations. - Finalizing vendor data /detailed engineering dependent fire case loads and finalizing corresponding relief valve inlet and outlet line sizes.</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>Page 17</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Cable trays / Junction Box</t>
+          <t>Telephone Intercom System</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Cable trays, Junction Box etc shall be of FRP / GRP material suitable for coastal region,</t>
+          <t>1.1 Manufacturer OR Vendor Service Assistance Where responsibility is not indicated in Section 2. a. Obtain the assistance of the manufacturer or vendor, when necessary, to make a satisfactory installation as agreed on by the LEPC Contractor and the Owner b. Obtain the assistance of the manufacturer or vendor, as required, for technical assistance during run-in by the training or for informational and operating purposes c. Furnish names and telephone numbers including emergency contact of manufacturers, and vendors, technical service representatives for use by the Owner.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Relevant to telecom/security cable containment where applicable.</t>
+          <t>Verbatim specification requirement extracted dynamically.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea</t>
+          <t>Part_B1_Technical_Specification_CO2_Urea_1_500</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>A. Technical Specification – Mechanical / 3.a Codes &amp; Standards-2</t>
+          <t>B773-000-16-43-TCL-9902, Preparation of specification for LEL, gas like hydrogen and ammonia detectors and providing the same at suitable locations. - Finalizing vendor data /detailed engineering dependent fire case loads and finalizing corresponding relief valve inlet and outlet line sizes.</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>Page 3</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Electrical installations / hazardous areas</t>
+          <t>Telecom Specifications</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>All electrical systems and installations shall comply with applicable IEC standards, including IEC 60079 series for hazardous areas, IEC 60364 for electrical installations, and IEC 60529 for ingress protection.</t>
+          <t>12 Bidder to confirm that technical requirements for purchase of piping items as per Engineering Design basis (Piping) – Doc. No. B773-000-16-43-EDB- 1001, EIL Piping &amp; Valve Material Specifications, General notes of EIL PMS &amp; VMS and Technical Notes for piping items are noted and understood. This shall be the basis for bidder’s detailed specification for procurement, as per Piping Scope of Supply &amp; Works, Doc. No. B773-000-16-43-SOW-9902. Bidder to confirm compliance.</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Relevant to telecom/security electrical installation and equipment protection.</t>
+          <t>Verbatim specification requirement extracted dynamically.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea</t>
+          <t>Part_B1_Technical_Specification_CO2_Urea_1_500</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>A. Technical Specification – Mechanical / 3.a Codes &amp; Standards-3</t>
+          <t>B773-000-16-51-SOW-9902, Preparation of specification for LEL, gas like hydrogen and ammonia detectors and providing the same at suitable locations. - Finalizing vendor data /detailed engineering dependent fire case loads and finalizing corresponding relief valve inlet and outlet line sizes.</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>Page 4</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Hazardous area / IP / coastal suitability</t>
+          <t>CCTV Surveillance System</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>The hydrogen generation plant shall be provided with electrical equipment and instrumentation suitable for installation in classified hazardous areas (Zone 1 and Zone 2) for Gas Group IIC (Hydrogen service), with appropriate temperature class. Outdoor equipment shall have minimum ingress protection of IP65/IP66, as applicable, and shall be designed with materials, surface treatments, and coatings suitable for the specified ambient and corrosive (coastal) environmental conditions.</t>
+          <t>2.2.6 CCTV system including Field mounted CCTV cameras with their cables, installation materials and accessories.</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Applies where telecom/security equipment is installed in hydrogen plant hazardous/coastal areas.</t>
+          <t>Verbatim specification requirement extracted dynamically.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea</t>
+          <t>Part_B1_Technical_Specification_CO2_Urea_1_500</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>A. Technical Specification – Mechanical / 3.b Design Considerations-5</t>
+          <t>B773-000-16-51-SOW-9902, Preparation of specification for LEL, gas like hydrogen and ammonia detectors and providing the same at suitable locations. - Finalizing vendor data /detailed engineering dependent fire case loads and finalizing corresponding relief valve inlet and outlet line sizes.</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>Page 5</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Remote operation / central control room</t>
+          <t>CCTV Surveillance System</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>The electrolyser package and associated hydrogen generation system shall be provided with adequate instrumentation, control, and automation features to enable safe remote operation, continuous monitoring, and supervisory control from the central control room.</t>
+          <t>SCOPE OF SUPPLY &amp; WORK (INSTRUMENTATION) 150 TPD GREEN UREA R&amp;D PROJECT, Client LTD Section-A.4.12 B773-000-16-51-SOW-9902 Rev. B Page 5 of 17 Template No. 5-0000-0001-T1 Rev. 1 Copyrights EIL – All rights reserved a) Distributed Control System (DCS) along with workstations, printers. b) Programmable logic controller (PLC) System for ESD and Interlocks, Fire &amp; Gas (F&amp;G), Package PLCs along with workstations, printers. c) CCTV System. d) Anti-surge / Performance Control System, Speed Governor Control System, Overspeed Protection System, Machine Monitoring System with workstations. e) Any other system oriented items. YES YES YES YES YES - - - - -</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Control/monitoring network and CCR integration relevance.</t>
+          <t>Verbatim specification requirement extracted dynamically.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea</t>
+          <t>Part_B1_Technical_Specification_CO2_Urea_1_500</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>A. Technical Specification – Mechanical / 4.b Design Considerations-7</t>
+          <t>B773-000-16-51-SOW-9902, Preparation of specification for LEL, gas like hydrogen and ammonia detectors and providing the same at suitable locations. - Finalizing vendor data /detailed engineering dependent fire case loads and finalizing corresponding relief valve inlet and outlet line sizes.</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>Page 8</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Remote monitoring / supervision / control</t>
+          <t>CCTV Surveillance System</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>The Cryogenic ASU shall be provided with adequate instrumentation, control, and automation features to enable safe local operation as well as remote monitoring, supervision, and control of nitrogen and oxygen production from the central control room.</t>
+          <t>2.4.4 Inspection and Testing of all field instruments, DCS/PLC System {including Package PLCs}, MMS, Anti-surge / Performance Control System, Speed Governor Control, Overspeed Protection System, Analysers, Gas Chromatograph, CCTV system, Local Control Panels etc as per Instrumentation Design Basis, Inspection Test Plans and other standard specifications, job specifications attached in the tender and respective instrumentation Purchase Requisitions.</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Control/monitoring network and CCR integration relevance.</t>
+          <t>Verbatim specification requirement extracted dynamically.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea</t>
+          <t>Part_B1_Technical_Specification_CO2_Urea_1_500</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>B. Technical Specification – Electrical / 7. ELECTRICAL / 5. Specific requirement for CO2 Capture Block / Item 5</t>
+          <t>B773-000-16-51-SOW-9902, Preparation of specification for LEL, gas like hydrogen and ammonia detectors and providing the same at suitable locations. - Finalizing vendor data /detailed engineering dependent fire case loads and finalizing corresponding relief valve inlet and outlet line sizes.</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>37</t>
+          <t>Page 9</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>DCS/PLC/Instrumentation Redundant UPS</t>
+          <t>CCTV Surveillance System</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>240V, 10kVA AC (Minimum) dual redundant with bypass UPS system (2 nos 1X100%) with Nickel cadmium battery, ACDB, cell booster for DCS/PLC/Instrumentation loads including spare feeders. Battery backup time of 3 hours.</t>
+          <t>2.5.4 Installation of DCS/ESD PLC system, CCTV System, MMS, Anti-surge / Performance Control System, Speed Governor Control, Overspeed Protection System, Package PLC based control system and related equipments, panels/cabinets, workstations, printers, any sub-package control system, cabinets and related accessories, supplied by Contractor. YES -</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Dual redundant 10kVA UPS system with Ni-Cd battery bank providing 3 hours backup for DCS/PLC and instrumentation loads at Site Alpha CO2 Capture Block.</t>
+          <t>Verbatim specification requirement extracted dynamically.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea</t>
+          <t>Part_B1_Technical_Specification_CO2_Urea_1_500</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>C. Technical Specification – Control &amp; Instrumentation / 8. CONTROL &amp; INSTRUMENTATION / 1 Hierarchy of Documents &amp; Overview / Clause 3</t>
+          <t>B773-000-16-51-SOW-9902, Preparation of specification for LEL, gas like hydrogen and ammonia detectors and providing the same at suitable locations. - Finalizing vendor data /detailed engineering dependent fire case loads and finalizing corresponding relief valve inlet and outlet line sizes.</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>38</t>
+          <t>Page 12</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Remote Monitoring &amp; Historian</t>
+          <t>CCTV Surveillance System</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>The bidder shall provide remote monitoring (read-only data flow) for the CO2 capture plant (located at Site Alpha) at Site Beta. The Site Beta standalone monitoring system shall be non-control, with no interface to plant control systems, and will follow cybersecurity-driven network isolation with secure, standardized communication (e.g., OPC) to ensure reliable data monitoring. The system shall include historian with a minimum storage capacity of two months.</t>
+          <t>SCOPE OF SUPPLY &amp; WORK (INSTRUMENTATION) 150 TPD GREEN UREA R&amp;D PROJECT, Client LTD Section-A.4.12 B773-000-16-51-SOW-9902 Rev. B Page 12 of 17 Template No. 5-0000-0001-T1 Rev. 1 Copyrights EIL – All rights reserved procurement, factory testing, site activities and site acceptance testing. b) Coordination with various vendors / other sub-contractors / manufacturers / sub packaged vendors etc associated with package instrument supplies and services. c) Coordination with suppliers of special instruments / instrumentation items, control systems (DCS/PLC), analysers, system oriented items (CCTV system, MMS System, Anti-surge / Performance Control System, Speed Governor Control, Overspeed Protection System, Package PLC etc.) for availability of their specialist persons during start up and commissioning of all the units. YES YES - -</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Establish a read-only remote monitoring interface from Site Alpha to Site Beta using OPC communication, including cybersecurity network isolation and a historian with minimum 2 months storage.</t>
+          <t>Verbatim specification requirement extracted dynamically.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea</t>
+          <t>Part_B1_Technical_Specification_CO2_Urea_1_500</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>C. Technical Specification – Control &amp; Instrumentation / 8. CONTROL &amp; INSTRUMENTATION / 1 Hierarchy of Documents &amp; Overview / Clause 4</t>
+          <t>B773-000-16-51-SOW-9902, Preparation of specification for LEL, gas like hydrogen and ammonia detectors and providing the same at suitable locations. - Finalizing vendor data /detailed engineering dependent fire case loads and finalizing corresponding relief valve inlet and outlet line sizes.</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>38</t>
+          <t>Page 13</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Cybersecurity Compliance</t>
+          <t>CCTV Surveillance System</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>The system shall comply with applicable cybersecurity standards like IEC 62443 and include redundant communication using managed switches.</t>
+          <t>2.11 Warranty for all Instrumentation items, Analysers/ GC, System oriented items like DCS/ PLC system, CCTV System, MMS System, Anti-surge / Performance Control System, Speed Governor Control, Overspeed Protection System, Package PLC etc.</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Mandatory cybersecurity compliance with IEC 62443 standard and network switch redundancy using managed switches.</t>
+          <t>Verbatim specification requirement extracted dynamically.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea</t>
+          <t>Part_B1_Technical_Specification_CO2_Urea_1_500</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>C. Technical Specification – Control &amp; Instrumentation / 8. CONTROL &amp; INSTRUMENTATION / 3 Design Considerations / Clause 4</t>
+          <t>B773-000-16-51-SOW-9902, Preparation of specification for LEL, gas like hydrogen and ammonia detectors and providing the same at suitable locations. - Finalizing vendor data /detailed engineering dependent fire case loads and finalizing corresponding relief valve inlet and outlet line sizes.</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>39</t>
+          <t>Page 13</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Remote Connectivity Security</t>
+          <t>CCTV Surveillance System</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Remote connectivity for the systems, limited to process viewing only. The bidder must supply the necessary hardware and software to enable remote connectivity, ensuring all required cyber security compliance is met as per IEC 62443.</t>
+          <t>2.12 CPWAMC: Comprehensive post warranty annual maintenance contract (to be quoted separately) for Contractor supplied DCS/ PLC System, Bagging/ weighing control system, Analysers ((except density, moisture, PH/conductivity), Gas Chromatograph, CCTV System, MMS and Package PLC System, Giant Screen. CPWAMC to be executed after expiry of warranty and shall be for 5 years duration for each item.</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Remote connections are restricted to process viewing only. Bidder must provide secure hardware/software for remote access compliant with IEC 62443.</t>
+          <t>Verbatim specification requirement extracted dynamically.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea</t>
+          <t>Part_B1_Technical_Specification_CO2_Urea_1_500</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>C. Technical Specification – Control &amp; Instrumentation / 8. CONTROL &amp; INSTRUMENTATION / 3 Design Considerations / Clause 5</t>
+          <t>B773-000-16-51-SOW-9902, Preparation of specification for LEL, gas like hydrogen and ammonia detectors and providing the same at suitable locations. - Finalizing vendor data /detailed engineering dependent fire case loads and finalizing corresponding relief valve inlet and outlet line sizes.</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>39</t>
+          <t>Page 13</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>System Log Retention</t>
+          <t>CCTV Surveillance System</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>System logs of all DCS/PLC infrastructure involved in the project shall be securely retained for a minimum period of 180 days to support audit and incident investigation requirements.</t>
+          <t>2.13 Training for Owner’s personnel: Contractor shall arrange Operation and Maintenance training for Owner’s personnel for Contractor supplied system oriented items like DCS/ PLC System, Analysers/ Gas chromatographs, CCTV system, MMS, Anti-surge / Performance Control System, Speed Governor Control, Overspeed Protection System, Package PLC, Bagging/Weighing Control System. The training shall include detail operation, configuration, modification, calibration,</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Secure storage and retention of system logs for all DCS/PLC network infrastructure for at least 180 days for security auditing.</t>
+          <t>Verbatim specification requirement extracted dynamically.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea</t>
+          <t>Part_B1_Technical_Specification_CO2_Urea_1_500</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>C. Technical Specification – Control &amp; Instrumentation / 8. CONTROL &amp; INSTRUMENTATION / 3 Design Considerations / Clause 6</t>
+          <t>B773-000-16-51-SOW-9902, Preparation of specification for LEL, gas like hydrogen and ammonia detectors and providing the same at suitable locations. - Finalizing vendor data /detailed engineering dependent fire case loads and finalizing corresponding relief valve inlet and outlet line sizes.</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>39-40</t>
+          <t>Page 15</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Password Access Control</t>
+          <t>CCTV Surveillance System</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>The system shall have built-in safety features that will allow/disallow certain functions and entry fields within a function to be under password control to protect against inadvertent and unauthorised use of these functions. Assignment of allowable functions and entry fields shall be on the basis of user profile. The system security shall contain various user levels with specific rights which shall be as finalized by the Employer during detailed engineering. However, no. of user levels, no. of users in a level and rights for each level shall be changeable by the programmer (Administrator). The rights of each user shall contain two types of privileges as follows: (a) Privileges for the DCS/PLC, (b) Privileges for the Operating System features. Typically following user levels shall be available: (a) Operator, (b) Supervisor, (c) Maintenance Engineer, (d) Programmer, (e) Shift /Station In charge.</t>
+          <t>5. Contractor shall carry out 3-D modelling, clash checking with other disciplines, including the following: - All line mounted/ equipment mounted instruments like control valves, on-off valves, safety valves, flow instruments, level instruments, temperature instruments, pressure instruments and accessories like fire-safe jacketing (if applicable), volume tanks etc. - Instrument cable ducts with fittings like elbows, tees, reducers etc. &amp; cable trays (of size ≥ 300mm) - Analyzer/GC shelters (if applicable), analyzer cabinets/ racks and other field racks/ panels/ cabinets, local control panels, etc - All types of junction boxes - Gas detectors with Hooters, Beacons - CCTV system field components - Instrument stanchions - Instrumentation ducts connectivity between main pipe rack &amp; all technical structures, heaters, compressors, major package skids, etc. - ESD Push button stations in field - For package units, where engineering is carried out by package vendor/ other agencies/ compressor package vendor- model free issued to contractor, modelling shall be carried out by contractor as a box with hook-up/ tie-in locations. Inside the box, it is the contractor’s responsibility to ensure that package vendor carries out the precise modelling. However during 90% model review contractor shall be responsible to superimpose the 3D model furnished by Package Vendors &amp; resolve any clashes with the main unit 3D model, as applicable.</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Role-based access control with password protection across different user levels (Operator, Supervisor, Maintenance, Programmer, Shift In charge) and separate privileges for DCS/PLC and OS.</t>
+          <t>Verbatim specification requirement extracted dynamically.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea</t>
+          <t>Part_B1_Technical_Specification_CO2_Urea_1_500</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>C. Technical Specification – Control &amp; Instrumentation / 8. CONTROL &amp; INSTRUMENTATION / 3 Design Considerations / Clause 7</t>
+          <t>B773-000-16-51-SOW-9902, Preparation of specification for LEL, gas like hydrogen and ammonia detectors and providing the same at suitable locations. - Finalizing vendor data /detailed engineering dependent fire case loads and finalizing corresponding relief valve inlet and outlet line sizes.</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>Page 15</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>Control system component redundancy</t>
+          <t>CCTV Surveillance System</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>The redundancy in control system components (Network Switches, Controller, Servers-if any, Power System, Prefab etc.) System shall be designed by the contractor to ensure that malfunction of any single Control system component/ power supply system component etc. shall not lead to loss of any major auxiliary or loss of control function or loss of protection function.</t>
+          <t>8. All field related support activities involved during pre-commissioning and commissioning including instrument re-calibration, valve stroke checking during logic checks, graphics check, complex loop checks, control loop schematics check etc. shall be in the scope of contractor. Arranging OEM visit to site during pre-commissioning and commissioning of Contractor supplied special instruments, valves, Nucleonic level instruments, systems oriented items like Analysers, Gas Chromatograph, DCS,PLC, MMS, CCTV system etc shall be provided by the contractor. Calibration of all Field Instruments, Control Valves, On/Off Valves, Safety Valves at site and checking during pre-commissioning and commissioning shall be in contractor’s scope. Contractor shall ensure that all instruments shall have valid calibration date before pre- commissioning and commissioning. Page 348 of 7525 : B773-000-83-41-LE-T-9902 : Rev. B</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>No single point of failure: redundant network switches, controllers, power supplies, and servers to ensure continuous control and protection.</t>
+          <t>Verbatim specification requirement extracted dynamically.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea</t>
+          <t>Part_B1_Technical_Specification_CO2_Urea_1_500</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>C. Technical Specification – Control &amp; Instrumentation / 8. CONTROL &amp; INSTRUMENTATION / 3 Design Considerations / Clause 8</t>
+          <t>B773-000-16-50-SOW-9902, Preparation of specification for LEL, gas like hydrogen and ammonia detectors and providing the same at suitable locations. - Finalizing vendor data /detailed engineering dependent fire case loads and finalizing corresponding relief valve inlet and outlet line sizes.</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>Page 6</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Conformal Coating</t>
+          <t>Telephone Intercom System</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>All the electronic modules PCB should have conformal coating that can provide protection against extreme moisture, corrosive gases and aggressive dust, or combinations thereof.</t>
+          <t>41. Main incoming telephone system junction box (TJB), Safe area telephone sets, telephone system cables from TJB onwards to safe area equipments within package battery limit. 3 3 3 3</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>Conformal coating on all electronic boards/PCBs to protect against coastal corrosion, humidity, and dust.</t>
+          <t>Verbatim specification requirement extracted dynamically.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea</t>
+          <t>Part_B1_Technical_Specification_CO2_Urea_1_500</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>C. Technical Specification – Control &amp; Instrumentation / 8. CONTROL &amp; INSTRUMENTATION / 3 Design Considerations / Clause 12</t>
+          <t>B773-000-16-50-SOW-9902, Preparation of specification for LEL, gas like hydrogen and ammonia detectors and providing the same at suitable locations. - Finalizing vendor data /detailed engineering dependent fire case loads and finalizing corresponding relief valve inlet and outlet line sizes.</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>Page 6</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>Network Hardening</t>
+          <t>Telephone Intercom System</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>Network infrastructure with firewall and cyber security and components shall be designed as per IEC 62443. System hardening must be ensured.</t>
+          <t>42. Power supply Feeders, cables, lighting fixtures etc. for beacon lamps, acoustic hoods, within package battery limit for plant communication and telephone system. 3 3 3 3</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>Network security requirements including firewall implementation, system hardening (disabling unused ports/services), and alignment with IEC 62443.</t>
+          <t>Verbatim specification requirement extracted dynamically.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea</t>
+          <t>Part_B1_Technical_Specification_CO2_Urea_1_500</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>C. Technical Specification – Control &amp; Instrumentation / 8. CONTROL &amp; INSTRUMENTATION / 3 Design Considerations / Clause 13</t>
+          <t>B773-000-16-50-SOW-9902, Preparation of specification for LEL, gas like hydrogen and ammonia detectors and providing the same at suitable locations. - Finalizing vendor data /detailed engineering dependent fire case loads and finalizing corresponding relief valve inlet and outlet line sizes.</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>Page 8</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>UPS Monitoring</t>
+          <t>Telephone Intercom System</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>UPS Systems monitoring signals to be hooked up with centralized DCS/PLC. Qty of signals shall be as recommended by OEM of UPS system.</t>
+          <t>52. All cable trays, cable ducts, supports, RCC cable trenches, conduits, within the package battery limit for all cables being supplied by contractor and all cables being supplied/ installed by owner for power, control, fire alarm, communication, telephone, ECS data highway and other systems. 3 3 3 3</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>Integration of UPS monitoring alarms and status signals with the central DCS/PLC system.</t>
+          <t>Verbatim specification requirement extracted dynamically.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea</t>
+          <t>Part_B1_Technical_Specification_CO2_Urea_1_500</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>C. Technical Specification – Control &amp; Instrumentation / 8. CONTROL &amp; INSTRUMENTATION / 3 Design Considerations / Clause 19</t>
+          <t>B773-000-16-50-SOW-9902, Preparation of specification for LEL, gas like hydrogen and ammonia detectors and providing the same at suitable locations. - Finalizing vendor data /detailed engineering dependent fire case loads and finalizing corresponding relief valve inlet and outlet line sizes.</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>Page 9</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>OS &amp; Anti-Virus Updates</t>
+          <t>Telephone Intercom System</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>The software packages including OS, Application software (eg GUI, History etc ) as per the functional requirement and Anti-Virus Software to be included with the Servers/Workstations/PC Stations (as applicable) shall also be the latest version available at the time of supply. As a customer support, the Contractor shall periodically inform and upgrade the Anti-Virus software of the workstations/servers/switches/firewall as applicable till completion of the warranty period and till the completion of the AMS period.</t>
+          <t>60. Preparation of equipment layouts, lighting layouts, cabling layouts, earthing layouts, lightning protection layout, NIFPS piping layout, plant communication layouts, fire alarm layouts, telephone layouts, LAN system layout, etc. 3 - - -</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>Supply latest software and OS versions. Provide periodic anti-virus engine and signature updates for workstations, servers, network switches, and firewalls during warranty and AMS.</t>
+          <t>Verbatim specification requirement extracted dynamically.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea</t>
+          <t>Part_B1_Technical_Specification_CO2_Urea_1_500</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>C. Technical Specification – Control &amp; Instrumentation / 8. CONTROL &amp; INSTRUMENTATION / 3 Design Considerations / Clause 20</t>
+          <t>B773-000-16-50-SOW-9902, Preparation of specification for LEL, gas like hydrogen and ammonia detectors and providing the same at suitable locations. - Finalizing vendor data /detailed engineering dependent fire case loads and finalizing corresponding relief valve inlet and outlet line sizes.</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>Page 9</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>History Server Redundancy</t>
+          <t>Telephone Intercom System</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>History function (Alarm/Event/Trend etc) for the units monitored and controlled from the operator console shall be dual redundant with each node having dual disc drives dedicated for history storage or with history storage available in each of the multiple operator stations of a console group.</t>
+          <t>61. Preparation of bill of materials for cabling, lighting, earthing and lightning protection, communication, plant communication, fire alarm, telephone system, LAN and miscellaneous items 3 - - -</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Dual redundant history logging (alarms, events, trends) using dedicated dual disk drives per node or distributed operator stations.</t>
+          <t>Verbatim specification requirement extracted dynamically.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea</t>
+          <t>Part_B1_Technical_Specification_CO2_Urea_1_500</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>C. Technical Specification – Control &amp; Instrumentation / 8. CONTROL &amp; INSTRUMENTATION / 4 Control System Architecture / Clause 1</t>
+          <t>B773-000-17-42-SOW-2501, Preparation of specification for LEL, gas like hydrogen and ammonia detectors and providing the same at suitable locations. - Finalizing vendor data /detailed engineering dependent fire case loads and finalizing corresponding relief valve inlet and outlet line sizes.</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>Page 4</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>DCS/PLC Processor Redundancy</t>
+          <t>Telephone Intercom System</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Centralized Controller shall be provided with Dual processor, Hot standby based DCS/PLC system (including main processing unit and memories) one for normal operation and one as hot standby – and should be suitably interfaced with HMI systems.</t>
+          <t>In case project activities are found to be delayed during the review, LEPC CONTRACTOR shall deploy additional resources over &amp; above the existing group. In case performance of any personnel deployed by LEPC CONTRACTOR under this project is found to be unsatisfactory by the Owner/ Consultant, the same shall be communicated to the CONTRACTOR for providing suitable replacement by CONTRACTOR within 07 (seven) days of communication by Owner / Consultant. e) During BDEP preparation, detailed Engineering, LEPC CONTRACTOR shall facilitate access for OWNER/PMC’s designated personnel at Licensor /Engineering subcontractor/LEPC contractor offices as required. LEPC CONTRACTOR shall provide office &amp; related office infrastructure facilities such as furniture, computer, courier service, telephone, email, Internet connectivity and Canteen facility for OWNER/PMC’s team during the aforesaid period. f) LEPC CONTRACTOR shall provide full assistance to OWNER and CONSULTANT’s personnel at all places during the course of the WORKS for the following: I. To enter into and go out from the countries. II. To stay in the countries for the required period. g) LEPC CONTRACTOR shall provide BDEP in accordance with requirements given in this bidding document. h) LEPC contractor will submit the consolidated effluent summary for effluents from all sources / facilities covered under LEPC contractor’s scope and provide treatment scheme. i) LEPC contractor shall provide overall water balance and provide the scheme for implementing Zero Liquid discharge philosophy. Approval on these documents are required to be obtained before submission of technical documents (design basis, technical specification, PFD P&amp;ID etc.) related to individual water and waste water treatment plant. j) LEPC contractor to ensure that any updation in water consumption / effluent generation are reflected in the updation of related documents and shall not have any bearing on design / turn down performance. All the units BEDP shall be revised by LEPC contractor based upon any such updation. k) LEPC CONTRACTOR shall provide engineering designs in accordance with BIDDING DOCUMENT, current worldwide best practices, the governing codes and in compliance with the Indian statutory regulations in force. l) LEPC CONTRACTOR shall submit all documents as per the agreed schedule. LEPC CONTRACTOR shall include drawings/documents listed elsewhere in BIDDING DOCUMENT as minimum requirements for submission to OWNER/PMC for approval or review or information. LEPC CONTRACTOR shall provide documentation keeping a review time by OWNER/PMC of fifteen (15) business working days to enable them Page 377 of 7525 : B773-000-83-41-LE-T-9902 : Rev. B</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>DCS/PLC controllers must feature dual processors with hot-standby redundancy for main processing units and memory.</t>
+          <t>Verbatim specification requirement extracted dynamically.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea</t>
+          <t>Part_B1_Technical_Specification_CO2_Urea_1_500</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>C. Technical Specification – Control &amp; Instrumentation / 8. CONTROL &amp; INSTRUMENTATION / 4 Control System Architecture / Clause 2</t>
+          <t>B773-000-17-42-SOW-2501, Preparation of specification for LEL, gas like hydrogen and ammonia detectors and providing the same at suitable locations. - Finalizing vendor data /detailed engineering dependent fire case loads and finalizing corresponding relief valve inlet and outlet line sizes.</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>Page 8</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>HMIPIS Network Interface</t>
+          <t>UPS &amp; DC Power Systems</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>Human - Machine Interface &amp; Plant Information System (HMIPIS): Minimum number of HMI PC Three (3)- OWS and One (1) EOWS, and one printer shall be provided for control room along with suitable console and furniture. The profile and dimension shall be decided during detailed engineering and shall be subject to Employer’s approval without any additional cost. PCs shall have Dual Ethernet interface with LAN accessories for all PC based OWS and EWS shall be provided. HMIPIS configured around latest state-of-the art servers/Workstations with open architecture supporting OPC/TCP/IP protocols, etc. shall be provided. This unified HMI can be interfaced either with the control systems of main plant or with propriety/native HMI of systems provided by OEM.</t>
+          <t>Copyright EIL – All rights reserved etc. as required and First Fill consumables. tt) Providing as built drawings /documents/ Vender doc/ Close out reports (Soft and Hard Copy). uu) LEPC contractor to ensure DCI/MCI connectivity with V-doc (Vendor Documentation portal) in each submission. vv) Document preparation &amp; submissions to be done by LEPC contractor only in the specified formats as specified elsewhere in the tender documents. ww) All online analyzers, Gas detectors, portable gas detector etc. located within ISBL are in LEPC contractors Scope. xx) LEPC Contractor shall update the Piping Material Specification (PMS) and Valve Material Specification (VMS) as per Process/Project requirements in-line with piping design basis and additional technical requirement and submit for Owner/PMC review. yy) LEPC Contractor shall update the welding specification charts based on requirements specified in ASME B 31.3, for classes not covered in Welding specification charts and for dissimilar material welding and submit it for review by Owner/ PMC. zz) Submission of in updated process package &amp; final documentation in state of art integrated documentation handover mode as specified elsewhere in tender document. aaa) Any other work required to complete the Process &amp; Utility systems and commission the units as per Process / Utility design requirements given in bid document and any other requirements given elsewhere in the tender document. bbb) Contractor to prepare battery limit interface based on given preliminary B/L interface and shall be submitted for Owner/PMC approval, preliminary B/L Interface details are as defined elsewhere in the bidding document. Page 381 of 7525 : B773-000-83-41-LE-T-9902 : Rev. B</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>Provide dual Ethernet network interfaces for all OWS and EWS PCs. System must use open architecture supporting OPC and TCP/IP.</t>
+          <t>Verbatim specification requirement extracted dynamically.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea</t>
+          <t>Part_B1_Technical_Specification_CO2_Urea_1_500</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>C. Technical Specification – Control &amp; Instrumentation / 8. CONTROL &amp; INSTRUMENTATION / 4 Control System Architecture / Clause 3</t>
+          <t>B773-000-16-43-SOW-9902, Common job specific Valve Material Specification for all the units/offsite covered in tender</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>41-42</t>
+          <t>Page 26</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>Large Video Screen Camera Integration</t>
+          <t>Telecom Specifications</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>The plant is envisaged to be controlled and monitored from the minimum two Large Video Screens (LVS) in association with its workstation mounted on the Unit Control Desk (UCD), located in the Central Common Control room under all regimes of operation i.e. start-up, shutdown, process control &amp; emergency handling i.e. suitable for plant operation. Large Video Screens (LVS) with its workstation (independent of OWS) and graphic processors to dynamically display plant data / mimics / alarms and any other process information. The Large Video screens shall have additional features to work in association with multiple numbers of plant cameras, if required, also to be supplied under this package.</t>
+          <t>5.4.20. VALVE MATERIAL SPECIFICATION Common job specific Valve Material Specification for all the units/offsite covered in tender shall be prepared by LEPC CONTRACTOR and same shall be submitted to OWNER / PMC for approval. Job specific VMS shall cover all Process/ Licensor’s material requirements, any additional requirements from OWNER/ PMC and shall be in line with EIL Valve material Specification B773-6-44-0006 provided with the tender. Any other VMS sheet required (other than detail VMS attached as document no. B773-6- 44-0006 during detail engineering to be developed by LEPC contractor. While developing valve material Specifications and requirements specified in Engineering design basis- Piping shall be followed. The valve material specification shall be developed on the similar format as EIL VMS format for each new type of valve and shall be submitted for review by OWNER / PMC. LEPC CONTRACTOR shall update the VMS as per comments (without any extra time &amp; cost to OWNER) and updated VMS shall be sent to OWNER/PMC for review/ records. Tests carried out on a particular size of one type of valve, pressure rating and material shall qualify all sizes equal to and below the test valve size for the same type, pressure rating and material. In case of austenitic SS, any one grade would qualify for all other grades of austenitic SS.</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>Integration of plant surveillance CCTV cameras with the control room Large Video Screens (LVS).</t>
+          <t>Verbatim specification requirement extracted dynamically.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea</t>
+          <t>Part_B1_Technical_Specification_CO2_Urea_1_500</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>C. Technical Specification – Control &amp; Instrumentation / 8. CONTROL &amp; INSTRUMENTATION / 4 Control System Architecture / Clause 4</t>
+          <t>B773-000-80-42-SOW-9902, specification for application of Torques and Hydraulic Bolt tension for flange joints, Document No. 6-76-0002”. LEPC CONTRACTOR shall calculate bolt tension and bolt torque values for the piping classes not covered in this specification and furnish the same</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>Page 5</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Controller Failover Time</t>
+          <t>Structured Cabling &amp; FOC</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>Centralized Controller shall have facility of bump less transfer in case of failure of one. In case of failure of working CPU, standby CPU shall takeover and maximum data loss shall be for 50ms.</t>
+          <t>b) Duly filled in equipment data sheets (approved copy) &amp; Performance curves (approved copy), for all cases. c) Duly-filled in experience record formats (approved copy) d) Equipment manufacturer's general reference list &amp; manufacturer's catalogue. e) List of Agreed Deviations (approved copy) f) Scope of supply / work, List of Mandatory spares, List of Commissioning spares, List of 2 years O&amp;M Spares and List of Special tools / tackles g) Site &amp; Utility Data / Specifications h) Applicable EDB, data sheets, job specifications, PMS/VMS, etc. of respective departments i) Utility data sheets j) Applicable Vendor list k) Applicable Painting Specifications, Site Spectra, etc. l) Detailed Vendor Data Requirements (i.e. GA drawing; C/S drawing; Layout drawing, P&amp;ID etc.) of all equipment &amp; components supplied by vendor. m) Applicable Owner/ PMC documents) n) Applicable Standards &amp; Specifications) o) Applicable Inspection Test Plan, etc.</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>Bumpless failover between redundant controller CPUs with maximum data loss limited to 50 milliseconds.</t>
+          <t>Verbatim specification requirement extracted dynamically.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea</t>
+          <t>Part_B1_Technical_Specification_CO2_Urea_1_500</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>C. Technical Specification – Control &amp; Instrumentation / 8. CONTROL &amp; INSTRUMENTATION / 4 Control System Architecture / Clause 5</t>
+          <t>B773-00-000-19-41, specification for application of Torques and Hydraulic Bolt tension for flange joints, Document No. 6-76-0002”. LEPC CONTRACTOR shall calculate bolt tension and bolt torque values for the piping classes not covered in this specification and furnish the same</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>Page 9</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>PLC SIL Level Study</t>
+          <t>Telephone Intercom System</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>SIL level of PLCs (standalone equipment/packages), instruments, solenoid valves etc. shall be decided as per HAZOP and SIL study.</t>
+          <t>CONSTRUCTION SUPERVISION AND MANAGEMENT BY LEPC FOR 150 TPD GREEN UREA COMPLEX OF Client DOCUMENT No. B773-00-000-19-41- 0002 Rev. 0 Page 9 of 23 Format No. EIL 1641-1924 Rev. 1 Copyright EIL – All rights reserved k. Mobile toilets and necessary arrangement for cleaning and disposal from refinery to outside refinery. l. Field Testing Laboratory m. Radiography Source Pit as per BARC Guidelines n. Film processing and viewing labs o. Communication facilities viz. Telephone, Fax, E-mail, electronic transmission of drawings./ documents, etc. p. Hutments, transport, Pantry and Canteen for staff and workers. Hutments/ labour colony shall not be allowed inside the refinery complex. q. Vehicle parking area including construction equipments. r. First aid arrangement/ medical and health care facilities s. Gate pass for workmen/officials/ vehicles as per OWNER security system. t. Work Permits as per Owner’s prevailing system. CONTRACTOR shall develop the temporary facilities layout for approval of Owner/PMC.</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>Safety Integrity Level (SIL) for package PLCs and field instrumentation must be determined through formal HAZOP and SIL studies.</t>
+          <t>Verbatim specification requirement extracted dynamically.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea</t>
+          <t>Part_B1_Technical_Specification_CO2_Urea_1_500</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>C. Technical Specification – Control &amp; Instrumentation / 8. CONTROL &amp; INSTRUMENTATION / 4 Control System Architecture / Clause 6</t>
+          <t>B773-00-000-19-41, specification for application of Torques and Hydraulic Bolt tension for flange joints, Document No. 6-76-0002”. LEPC CONTRACTOR shall calculate bolt tension and bolt torque values for the piping classes not covered in this specification and furnish the same</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>Page 19</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>UPS Redundancy &amp; Backup</t>
+          <t>Telecom Specifications</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>All C&amp;I System including PLC along with OWS (Operator Workstation) &amp; EWS (Engineers Workstation), Analyzers, instruments etc. shall be powered by Redundant UPS (2 X 100 %) along with battery backup in accordance with Electrical specifications. System must be supplied with at least two-hour backup.</t>
+          <t>CONSTRUCTION SUPERVISION AND MANAGEMENT BY LEPC FOR 150 TPD GREEN UREA COMPLEX OF Client DOCUMENT No. B773-00-000-19-41- 0002 Rev. 0 Page 19 of 23 Format No. EIL 1641-1924 Rev. 1 Copyright EIL – All rights reserved CONTRACTOR shall be completely responsible for management of approved quality plans and Owner/PMC involvement will be only of Surveillance in nature to randomly check the works at selective/critical junctures. Their role shall be to monitor that the CONTRACTOR is executing the quality plans as per the approved drawings, employing adequately qualified staff and other resources for various items of works. Any deviation to the specifications shall be brought to the notice of Owner/PMC in prescribed formats by CONTRACTOR for approval. (ii) It is likely that the CONTRACTOR may engage sub-contractor(s)/vendors for performance of the work. CONTRACTOR shall be responsible for ensuring the implementation of approved QA plan, contract specifications and contract conditions through their sub-contractors to achieve the quality during all stages of construction. It shall be the responsibility of the CONTRACTOR to ensure proper coordination between his sub- contractor(s) and other agencies working at site. The sub-contractor(s)/vendors selection shall be done after evaluation by the CONTRACTOR in line with contract requirements and shall be got approved by Owner/PMC before engaging them for the works. (iii) Storage All the materials procured shall be stored/stacked as per the standard norms and as recommended in various clauses of relevant codes and contract document. The storage of material shall be such as to avoid damage to life/properties (physical and chemical) of the materials. The storage shall not cause deterioration, rusting, mix-up etc. and hamper the other related works in any way. CONTRACTOR shall submit his detailed warehouse plan for Owner/PMC approval to manage the above in open/covered areas. The materials susceptible to fire shall be kept away in a separate protected place. In general, the materials shall be kept systematically in order of their class, batch number and identification number, so that they are accessible for the inspection by Owner/PMC whenever required and to avoid the mix up in those materials. (iv) Use The materials shall be stacked in such a way that the lot, which is procured first, will be consumed first. For materials which are having specific expiry date/ shelf life shall not be used beyond that date and shall be removed from site. Wherever there is any doubt about the change in properties of the materials, such materials shall be sent to reputed approved laboratory for testing and acceptance. (v) Inspection The CONTRACTOR shall be responsible for carrying out inspection of the materials brought at site and conducting tests/ checks (at site or in approved laboratories) at predefined frequencies as per contract. It is the responsibility of the CONTRACTOR to ensure that the materials used at site shall conform to relevant codes/ standards and Manufacturer Test Certificates are available for correlation as and when required. The CONTRACTOR shall maintain the records of all materials brought at site and tests conducted on them. (vi) In process and final Inspection CONTRACTOR shall be responsible to arrange verification of products during in- process and final inspection. Relevant checks and tests shall be arranged for the works performed and records maintained. Tolerances achieved with respect to contract specification and execution drawings for various activities/processes shall be ascertained and submitted to Owner/PMC for approval. Efforts shall be made to keep checks and controls in such a way that a non-conforming product is avoided. However, if in an isolated case, the tolerances are beyond the acceptable values given in the contract/execution drawings/codes, non- Page 460 of 7525 : B773-000-83-41-LE-T-9902 : Rev. B</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>Provide dual redundant 2x100% UPS system with minimum 2-hour battery backup for all C&amp;I systems, PLCs, OWS/EWS, and analyzers.</t>
+          <t>Verbatim specification requirement extracted dynamically.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea</t>
+          <t>Part_B1_Technical_Specification_CO2_Urea_1_500</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>C. Technical Specification – Control &amp; Instrumentation / 8. CONTROL &amp; INSTRUMENTATION / 4 Control System Architecture / Clause 7</t>
+          <t>B773-000-83-41-LE-T-9902, Specification for Health, Safety and Environment (HSE) Management (Spec. No. 6-82-0001) is required to be followed by CONTRACTOR during Construction Phase at site. 2.0 CONTRACTOR shall have a documented HSE policy to cover commitment of the organization to ensure Health, Safety and Environment aspects in the line of operation.</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>471</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Redundant Communication Bus</t>
+          <t>Telecom Specifications</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>Data Communication System Bus connecting Control System and HMIPIS. Other bus systems for connecting various systems/subsystems like Cubicle Bus, Local Bus, I/O Bus (Including Remote I/O Bus) soft links (including those from Field Bus based temperature transmitter) as well as within systems/sub-systems. All the bus systems shall be redundant except for backplane buses which can be non-redundant.</t>
+          <t>2. Contractor to submit job procedures for the jobs for which ITP’s are attached &amp; job specific reporting formats with the aid of enclosed sample reporting formats to EIL/Owner for approval, before commencement of the activity. If the contractor has to deviate from the given ITP for a valid reason, he shall obtain prior written approval of EIL/Owner. Contractor to carry out 100% examination of all activities. LEGEND HP : Hold Point ; An activity which requires witnessing/inspection/verification and acceptance by Owner/EIL before any further processing is permitted. The Contractor shall not process the activity/item beyond a Hold Point without written approval by Owner/EIL except where prior written permission for further processing is available. WwW : Witness Point ; An activity which requires witnessing/inspection/verification by Owner/EIL when the activity is performed. After proper notification has been provided (notification modalities and period shall be finalized before hand), the Contractor is not obliged to hold further processing if Owner/EIL is not available to witness the activity or does not provide comments before the date notified. Basis of acceptance shall be on review of Contractor generated report/document as per relevant technical specification. Rw : Review of Contractor’s documentation. S : Surveillance Inspection by Owner/ EIL. Monitoring or making observations to verify whether or not material/items or services conform to specified requirements. Surveillance activities may include audit, inspections, witness of testing, Review of quality documentation &amp; records, personnel qualifications, etc. WC se: 100% Supervision and Examination by Contractor. Responsibility for execution of the inspection/testing is with the Contractor; Owner/EIL only verifies examination or testing done by the Contractor at important stages. Format No. 8-00-0001-F1 Rev. 0 Copyright EIL — All rights reserved Paaqe 471 of 7525 - B773-000-83-41-L E-T-9902 -Rev.B</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>Redundant system communication buses connecting control systems and HMIPIS, including I/O and cubicle buses.</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="2" t="inlineStr">
-        <is>
-          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea</t>
-        </is>
-      </c>
-      <c r="B30" s="2" t="inlineStr">
-        <is>
-          <t>C. Technical Specification – Control &amp; Instrumentation / 8. CONTROL &amp; INSTRUMENTATION / 4 Control System Architecture / Clause 8</t>
-        </is>
-      </c>
-      <c r="C30" s="3" t="inlineStr">
-        <is>
-          <t>42</t>
-        </is>
-      </c>
-      <c r="D30" s="2" t="inlineStr">
-        <is>
-          <t>Sequence of Events Recording</t>
-        </is>
-      </c>
-      <c r="E30" s="2" t="inlineStr">
-        <is>
-          <t>Sequence of events recording function for with a resolution of one millisecond with facility of historical storage.</t>
-        </is>
-      </c>
-      <c r="F30" s="2" t="inlineStr">
-        <is>
-          <t>Sequence of Events Recording (SOER) capability with 1-millisecond resolution for event/alarm analysis.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="2" t="inlineStr">
-        <is>
-          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea</t>
-        </is>
-      </c>
-      <c r="B31" s="2" t="inlineStr">
-        <is>
-          <t>C. Technical Specification – Control &amp; Instrumentation / 8. CONTROL &amp; INSTRUMENTATION / 4 Control System Architecture / Clause 9</t>
-        </is>
-      </c>
-      <c r="C31" s="3" t="inlineStr">
-        <is>
-          <t>42</t>
-        </is>
-      </c>
-      <c r="D31" s="2" t="inlineStr">
-        <is>
-          <t>Field Instrument Ingress Protection</t>
-        </is>
-      </c>
-      <c r="E31" s="2" t="inlineStr">
-        <is>
-          <t>All electronic instruments and enclosures in field shall be dust proof and weatherproof to IP-65 as per IEC-60529 or equivalent NEMA enclosure rating or better and secure against the ingress of fumes, dampness, insects, and vermin. All external surfaces shall be suitably treated to provide protection against corrosive plant atmosphere.</t>
-        </is>
-      </c>
-      <c r="F31" s="2" t="inlineStr">
-        <is>
-          <t>IP65 minimum rating for field instruments, with protection against humidity, dust, vermin, and corrosive coastal atmosphere.</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea</t>
-        </is>
-      </c>
-      <c r="B32" s="2" t="inlineStr">
-        <is>
-          <t>C. Technical Specification – Control &amp; Instrumentation / 8. CONTROL &amp; INSTRUMENTATION / 4 Control System Architecture / Clause 11</t>
-        </is>
-      </c>
-      <c r="C32" s="3" t="inlineStr">
-        <is>
-          <t>42</t>
-        </is>
-      </c>
-      <c r="D32" s="2" t="inlineStr">
-        <is>
-          <t>Coastal Cable Trays &amp; Enclosures</t>
-        </is>
-      </c>
-      <c r="E32" s="2" t="inlineStr">
-        <is>
-          <t>The Control and Instrumentation (C&amp;I) system including conduits / cable sub trays / cabling accessories/ impulse piping / air supply piping / local instrument enclosures and racks/ accessories etc shall be designed in accordance with standards suitable for coastal environments, taking into account factors such as high humidity, salinity, and corrosion potential. All equipment and components must comply with relevant international standards such as IEC, IEEE, and NEMA, with materials and enclosures rated for marine or coastal use (e.g., stainless steel 316, IP66/NEMA 4X). Appropriate protective measures, including conformal coating, sealing, and environmental shielding and the use of corrosion-resistant paints etc. shall be implemented to ensure reliable and long-term operation.</t>
-        </is>
-      </c>
-      <c r="F32" s="2" t="inlineStr">
-        <is>
-          <t>C&amp;I containment, conduits, racks, and local enclosures must be marine-grade (SS316, IP66, NEMA 4X) to resist coastal salinity and humidity.</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="2" t="inlineStr">
-        <is>
-          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea</t>
-        </is>
-      </c>
-      <c r="B33" s="2" t="inlineStr">
-        <is>
-          <t>C. Technical Specification – Control &amp; Instrumentation / 8. CONTROL &amp; INSTRUMENTATION / 4 Control System Architecture / Clause 12</t>
-        </is>
-      </c>
-      <c r="C33" s="3" t="inlineStr">
-        <is>
-          <t>43</t>
-        </is>
-      </c>
-      <c r="D33" s="2" t="inlineStr">
-        <is>
-          <t>CCTV Surveillance System</t>
-        </is>
-      </c>
-      <c r="E33" s="2" t="inlineStr">
-        <is>
-          <t>The CCTV System for monitoring of area along with all its components, i.e. necessary hardware and software, interface to the LVS of HMIPIS, the nos. of camera units, servers, network video recorder, network switches, modules and software, any other hardware/ software required for the safe and satisfactory operation, control, protection, monitoring, testing and maintenance of the system shall be provided by the Bidder. The system operation would be covering the complete view of the areas with pan / tilt, zoom, propositioning of the cameras and with programmability to monitor any camera on any monitor either manually or automatically in a defined switching. All cameras shall have CE/FCC/UL/BIS/STQC certification with consideration that cameras shall meet or exceed the statutory requirements as per applicable government norms. The server memory needs to be sufficient for storage of 2 months minimum. The total Camera quantity shall be minimum 20 Nos. Including 12 nos. for outdoor and 08 nos. for indoor. The final number of cameras shall not be limited to the quantities mentioned above. Vendor MUST note that the exact quantity and type (indoor/outdoor) shall be finalized during the detailed engineering, based on site conditions, surveillance coverage requirements without any extra cost to employer.</t>
-        </is>
-      </c>
-      <c r="F33" s="2" t="inlineStr">
-        <is>
-          <t>IP-based CCTV system with NVR storage of at least 2 months and a minimum camera count of 20 (12 outdoor, 8 indoor).</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="2" t="inlineStr">
-        <is>
-          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea</t>
-        </is>
-      </c>
-      <c r="B34" s="2" t="inlineStr">
-        <is>
-          <t>C. Technical Specification – Control &amp; Instrumentation / 8. CONTROL &amp; INSTRUMENTATION / 4 Control System Architecture / Clause 13</t>
-        </is>
-      </c>
-      <c r="C34" s="3" t="inlineStr">
-        <is>
-          <t>43</t>
-        </is>
-      </c>
-      <c r="D34" s="2" t="inlineStr">
-        <is>
-          <t>IP Public Address System (PAGA)</t>
-        </is>
-      </c>
-      <c r="E34" s="2" t="inlineStr">
-        <is>
-          <t>IP Based Public Address system including Call stations, loudspeakers, Network switches, Servers, PA system management Software &amp; other applicable software(s), PC Stations, Interconnecting cable etc. for all the units, common plant areas shall be provided by the Contractor. Minimum Quantity of Master Control Unit (MCU)- 1 nos. (in Centralized Control room), Indoor type calling stations- 3 nos. (with amplifier and loudspeaker), Outdoor type calling station- 5 nos. (with amplifier and loudspeaker), Acoustic hood- 2 nos., All the other items- hardware, software, licenses, including public address system erection hardware, all type of cables, cable tray, junction boxes, racks, conduits, etc. as required for the proper installation (conforming to IS:1881, IS:1882) to make the IP based PA system complete and functional are under Contractor's scope on as required basis.Vendor MUST note that the exact quantity of components shall be finalized during the detailed engineering, based on site conditions , system coverage requirements without any extra cost to employer.</t>
-        </is>
-      </c>
-      <c r="F34" s="2" t="inlineStr">
-        <is>
-          <t>IP-based PAGA system with 1 Master Control Unit in CCR, 3 indoor and 5 outdoor call stations, and 2 acoustic hoods, meeting IS:1881/1882.</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="2" t="inlineStr">
-        <is>
-          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea</t>
-        </is>
-      </c>
-      <c r="B35" s="2" t="inlineStr">
-        <is>
-          <t>C. Technical Specification – Control &amp; Instrumentation / 8. CONTROL &amp; INSTRUMENTATION / 4 Control System Architecture / Clause 14</t>
-        </is>
-      </c>
-      <c r="C35" s="3" t="inlineStr">
-        <is>
-          <t>43</t>
-        </is>
-      </c>
-      <c r="D35" s="2" t="inlineStr">
-        <is>
-          <t>GPS Clock Synchronization</t>
-        </is>
-      </c>
-      <c r="E35" s="2" t="inlineStr">
-        <is>
-          <t>Master &amp; Slave Clock System: One Geo-positionary satellite (GPS) based Master Clock in redundant configuration and slave clock for main plant and common areas shall be provided with suitable equipment including antenna, receiver and associated electronics to receive synchronization signals from GPS. The master clock shall synchronize all the systems (main and subsystem/standalone) at suitable intervals to maintain uniform time throughout the CO2 capture plant as per requirement.</t>
-        </is>
-      </c>
-      <c r="F35" s="2" t="inlineStr">
-        <is>
-          <t>Redundant GPS Master Clock and slave clocks to synchronize time across all control and network systems.</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="2" t="inlineStr">
-        <is>
-          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea</t>
-        </is>
-      </c>
-      <c r="B36" s="2" t="inlineStr">
-        <is>
-          <t>C. Technical Specification – Control &amp; Instrumentation / 8. CONTROL &amp; INSTRUMENTATION / 4 Control System Architecture / Clause 15</t>
-        </is>
-      </c>
-      <c r="C36" s="3" t="inlineStr">
-        <is>
-          <t>43</t>
-        </is>
-      </c>
-      <c r="D36" s="2" t="inlineStr">
-        <is>
-          <t>Separate Power Supply Bus</t>
-        </is>
-      </c>
-      <c r="E36" s="2" t="inlineStr">
-        <is>
-          <t>Separate power supply bus shall be provided for interrogation voltage supply for all inputs and output respectively (even if the input interrogation voltage and output voltage is same).</t>
-        </is>
-      </c>
-      <c r="F36" s="2" t="inlineStr">
-        <is>
-          <t>Isolate inputs and outputs by providing separate interrogation voltage power supply buses.</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="2" t="inlineStr">
-        <is>
-          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea</t>
-        </is>
-      </c>
-      <c r="B37" s="2" t="inlineStr">
-        <is>
-          <t>C. Technical Specification – Control &amp; Instrumentation / 8. CONTROL &amp; INSTRUMENTATION / 4 Control System Architecture / Clause 16</t>
-        </is>
-      </c>
-      <c r="C37" s="3" t="inlineStr">
-        <is>
-          <t>44</t>
-        </is>
-      </c>
-      <c r="D37" s="2" t="inlineStr">
-        <is>
-          <t>DCS/PLC Maintenance Training</t>
-        </is>
-      </c>
-      <c r="E37" s="2" t="inlineStr">
-        <is>
-          <t>Training (Minimum 7 days) for troubleshooting, maintenance and modification of centralized DCS/PLC and package PLCs-if any.</t>
-        </is>
-      </c>
-      <c r="F37" s="2" t="inlineStr">
-        <is>
-          <t>Minimum 7 days of technical training for plant staff covering troubleshooting, maintenance, and modification of the DCS and PLCs.</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="2" t="inlineStr">
-        <is>
-          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea</t>
-        </is>
-      </c>
-      <c r="B38" s="2" t="inlineStr">
-        <is>
-          <t>C. Technical Specification – Control &amp; Instrumentation / 8. CONTROL &amp; INSTRUMENTATION / 4 Control System Architecture / Clause 17</t>
-        </is>
-      </c>
-      <c r="C38" s="3" t="inlineStr">
-        <is>
-          <t>44</t>
-        </is>
-      </c>
-      <c r="D38" s="2" t="inlineStr">
-        <is>
-          <t>Sub-package communication link</t>
-        </is>
-      </c>
-      <c r="E38" s="2" t="inlineStr">
-        <is>
-          <t>All sub packages with its utilities shall be connected to centralized control room PLC through a two-way communication link.</t>
-        </is>
-      </c>
-      <c r="F38" s="2" t="inlineStr">
-        <is>
-          <t>Bidder must establish two-way communication links between all package/utility PLCs and the centralized DCS/PLC.</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="2" t="inlineStr">
-        <is>
-          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea</t>
-        </is>
-      </c>
-      <c r="B39" s="2" t="inlineStr">
-        <is>
-          <t>C. Technical Specification – Control &amp; Instrumentation / 8. CONTROL &amp; INSTRUMENTATION / 4 Control System Architecture / Clause 18</t>
-        </is>
-      </c>
-      <c r="C39" s="3" t="inlineStr">
-        <is>
-          <t>44</t>
-        </is>
-      </c>
-      <c r="D39" s="2" t="inlineStr">
-        <is>
-          <t>Integration signals</t>
-        </is>
-      </c>
-      <c r="E39" s="2" t="inlineStr">
-        <is>
-          <t>For integration purposes the contractor shall determine all the optimal hardwire and soft signals required to achieve data transfer for integration purposes and hence collect this data.</t>
-        </is>
-      </c>
-      <c r="F39" s="2" t="inlineStr">
-        <is>
-          <t>Identify and implement appropriate hardwired and software-based data interfaces for system integration.</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="2" t="inlineStr">
-        <is>
-          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea</t>
-        </is>
-      </c>
-      <c r="B40" s="2" t="inlineStr">
-        <is>
-          <t>C. Technical Specification – Control &amp; Instrumentation / 8. CONTROL &amp; INSTRUMENTATION / 4 Control System Architecture / Clause 19</t>
-        </is>
-      </c>
-      <c r="C40" s="3" t="inlineStr">
-        <is>
-          <t>44</t>
-        </is>
-      </c>
-      <c r="D40" s="2" t="inlineStr">
-        <is>
-          <t>Centralized Controller protocol interface</t>
-        </is>
-      </c>
-      <c r="E40" s="2" t="inlineStr">
-        <is>
-          <t>Centralized Controller must be able to get interface with other PLC as per the future requirements via Ethernet or Modbus RS 485 protocol.</t>
-        </is>
-      </c>
-      <c r="F40" s="2" t="inlineStr">
-        <is>
-          <t>Centralized controllers must support standard Modbus RS485 and Ethernet communication protocols for interfacing with external PLCs.</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="2" t="inlineStr">
-        <is>
-          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea</t>
-        </is>
-      </c>
-      <c r="B41" s="2" t="inlineStr">
-        <is>
-          <t>Technical Specifications: Part-A / Section M: Civil / 5 Buildings &amp; Structures / Item (iii)</t>
-        </is>
-      </c>
-      <c r="C41" s="3" t="inlineStr">
-        <is>
-          <t>47</t>
-        </is>
-      </c>
-      <c r="D41" s="2" t="inlineStr">
-        <is>
-          <t>Control Room Civil Design - Site Alpha</t>
-        </is>
-      </c>
-      <c r="E41" s="2" t="inlineStr">
-        <is>
-          <t>Electrical cum Control Room for Carbon capture plant at Site Alpha: A RCC / pre-engineered structural steel Building (25m X 12m) tentative shall be provided. The building shall be covered from all sides. The Electrical Room shall accommodate, LT PMCC Panels, Dry Type Transformer (if applicable), VFD Transformers (if applicable), 220V DCFB, LDB, WDB. and UPS, UPS DCDB, UPS battery and operator cabin etc. as per functional requirement. However, final size of Switchgear room, Control room, individual room, partition, doors, windows, rolling shutter etc shall be finalized at the stage of detail engineering with the approval of Client. Control room, meeting room, office space with toilet, pantry, staircase etc., shall be provided with sufficient lighting, ceiling / wall mounted fans, office furniture (tables, chairs etc of reputed make) etc. Individual control room, meeting room, office space shall be able to house 5-8 people for regular operational requirement. Control Room shall be Air conditioned. The control shall accommodate all the equipment as mentioned in Electrical and C&amp;I chapter. The firefighting system shall be provided as per norms.</t>
-        </is>
-      </c>
-      <c r="F41" s="2" t="inlineStr">
-        <is>
-          <t>Tentative 25x12m air-conditioned building at Site Alpha to house C&amp;I and electrical systems, including UPS systems, batteries, and the operator cabin.</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="2" t="inlineStr">
-        <is>
-          <t>Part_A_Technical_Specification_150_TPD_CO2_To_Urea</t>
-        </is>
-      </c>
-      <c r="B42" s="2" t="inlineStr">
-        <is>
-          <t>Technical Specifications: Part-A / Section M: Civil / 5 Buildings &amp; Structures / Item (iv)</t>
-        </is>
-      </c>
-      <c r="C42" s="3" t="inlineStr">
-        <is>
-          <t>47</t>
-        </is>
-      </c>
-      <c r="D42" s="2" t="inlineStr">
-        <is>
-          <t>Control Room Civil Design - Site Beta</t>
-        </is>
-      </c>
-      <c r="E42" s="2" t="inlineStr">
-        <is>
-          <t>Electrical cum Control Room for Urea Plant at Site Beta shall be as mentioned in technical Specification (Part-B). Bidder shall be free to locate civil structures including control room in a manner to avoid blast proof constructions. Client...</t>
-        </is>
-      </c>
-      <c r="F42" s="2" t="inlineStr">
-        <is>
-          <t>Site Beta Control Room civil design specification, with layout flexibility to avoid blast-proof construction while maintaining OISD compliance.</t>
+          <t>Verbatim specification requirement extracted dynamically.</t>
         </is>
       </c>
     </row>

</xml_diff>